<commit_message>
feat(test): add comprehensive test suite for user management via Excel
- Integrated Excel data-driven testing for login and registration.
- Added Positive Login, Negative Login, and E2E Registration scenarios.
- Implemented RegistrationPage using Page Object Model (POM).
- Standardized error messages and logs in English.
- Optimized Driver and Hooks for stable browser lifecycle management.
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18255" windowHeight="10980"/>
+    <workbookView windowWidth="19770" windowHeight="11700"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -35,10 +35,34 @@
     <t>password</t>
   </si>
   <si>
+    <t>name</t>
+  </si>
+  <si>
     <t>ahmet.qa.at@gamil.com</t>
   </si>
   <si>
     <t>SecurePass123</t>
+  </si>
+  <si>
+    <t>Ahmet</t>
+  </si>
+  <si>
+    <t>user2@test.com</t>
+  </si>
+  <si>
+    <t>WrongPass456</t>
+  </si>
+  <si>
+    <t>WrongUser</t>
+  </si>
+  <si>
+    <t>test_user_unique_1@mail.com</t>
+  </si>
+  <si>
+    <t>SecurePass789</t>
+  </si>
+  <si>
+    <t>NewUser</t>
   </si>
 </sst>
 </file>
@@ -675,7 +699,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -687,6 +711,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1221,28 +1251,61 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:2">
+    <row r="1" ht="15.75" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" ht="29.25" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2" ht="29.25" spans="1:3">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="ahmet.qa.at@gamil.com"/>
+    <hyperlink ref="A3" r:id="rId2" display="user2@test.com"/>
+    <hyperlink ref="A4" r:id="rId3" display="test_user_unique_1@mail.com" tooltip="mailto:test_user_unique_1@mail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>